<commit_message>
feat: implementar verificador publico de certificados OS-10 con QR, simulador de franquicia SENCE para empresas y aula virtual interactiva con simulador de examen en LMS
</commit_message>
<xml_diff>
--- a/Carta_Gantt_PrevySeg_2026.xlsx
+++ b/Carta_Gantt_PrevySeg_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="357">
   <si>
     <t>PREVYSEG 2026 — CRONOGRAMA MAESTRO Y CARTA GANTT (1 MES / 30 DÍAS + EXTENSIONES)</t>
   </si>
@@ -975,22 +975,40 @@
     <t>Información transparente de costos, códigos SENCE y matrículas directas para personas y empresas.</t>
   </si>
   <si>
-    <t>v1.9.0 (Futuro)</t>
-  </si>
-  <si>
-    <t>Backend API / Base de Datos</t>
-  </si>
-  <si>
-    <t>Próxima Iteración</t>
-  </si>
-  <si>
-    <t>Conexión a base de datos PostgreSQL, pasarela de pagos Webpay y generación de certificados con código QR.</t>
-  </si>
-  <si>
-    <t>Automatización total de matrículas y validación pública de alumnos.</t>
-  </si>
-  <si>
-    <t>Plataforma 100% autoservicio.</t>
+    <t>v1.9.0</t>
+  </si>
+  <si>
+    <t>src/components/CertificateVerifierModal.jsx, SenceCalculatorModal.jsx, lms/views/CourseClassroomView.jsx</t>
+  </si>
+  <si>
+    <t>Nuevas Features / LMS &amp; B2B</t>
+  </si>
+  <si>
+    <t>Implementación del Verificador Público de Certificados OS-10 con QR, Simulador de Franquicia SENCE 100% y Cotizador Formal PDF para empresas, y Aula Virtual interactiva con reproductor de clases, temarios y simulador de examen teórico OS-10.</t>
+  </si>
+  <si>
+    <t>Aumentar la conversión comercial B2B, dar validación legal inmediata a egresados y enriquecer la experiencia educativa del estudiante en el campus virtual.</t>
+  </si>
+  <si>
+    <t>Plataforma líder en el norte de Chile con verificación en tiempo real, autoservicio corporativo y aula virtual interactiva.</t>
+  </si>
+  <si>
+    <t>v2.0.0 (Futuro)</t>
+  </si>
+  <si>
+    <t>Backend API / Base de Datos / Webpay</t>
+  </si>
+  <si>
+    <t>Próxima Iteración Mayor</t>
+  </si>
+  <si>
+    <t>Conexión a base de datos PostgreSQL en producción, pasarela de pagos Webpay Plus en cuotas y webhook de matriculación automática.</t>
+  </si>
+  <si>
+    <t>Automatización total de pagos en línea y alta disponibilidad.</t>
+  </si>
+  <si>
+    <t>Ecosistema 100% autosuficiente y transaccional.</t>
   </si>
   <si>
     <t>En Planificación</t>
@@ -5332,7 +5350,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -5622,7 +5640,7 @@
         <v>313</v>
       </c>
       <c r="B13" s="74" t="s">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C13" s="73" t="s">
         <v>314</v>
@@ -5639,8 +5657,34 @@
       <c r="G13" s="73" t="s">
         <v>318</v>
       </c>
-      <c r="H13" s="78" t="s">
+      <c r="H13" s="72" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="76" t="s">
         <v>319</v>
+      </c>
+      <c r="B14" s="71" t="s">
+        <v>241</v>
+      </c>
+      <c r="C14" s="70" t="s">
+        <v>320</v>
+      </c>
+      <c r="D14" s="71" t="s">
+        <v>321</v>
+      </c>
+      <c r="E14" s="70" t="s">
+        <v>322</v>
+      </c>
+      <c r="F14" s="70" t="s">
+        <v>323</v>
+      </c>
+      <c r="G14" s="70" t="s">
+        <v>324</v>
+      </c>
+      <c r="H14" s="78" t="s">
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -5667,7 +5711,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="67" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="B1" s="67"/>
       <c r="C1" s="67"/>
@@ -5677,104 +5721,104 @@
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="79" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="B3" s="79" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="C3" s="79" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="D3" s="79" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="E3" s="79" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="80" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="B4" s="81" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="C4" s="70" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="D4" s="70" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="E4" s="70" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="82" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="B5" s="83" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="C5" s="73" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="D5" s="73" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="E5" s="73" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="80" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="B6" s="81" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="C6" s="70" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="D6" s="70" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="82" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="B7" s="83" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="C7" s="73" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="D7" s="73" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="E7" s="73" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="80" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="B8" s="81" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="C8" s="70" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="D8" s="70" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="E8" s="70" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: integrar seccion de tramos SENCE en inicio y panel de visto bueno administrativo para emision de certificados sin notas confidenciales
</commit_message>
<xml_diff>
--- a/Carta_Gantt_PrevySeg_2026.xlsx
+++ b/Carta_Gantt_PrevySeg_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="363">
   <si>
     <t>PREVYSEG 2026 — CRONOGRAMA MAESTRO Y CARTA GANTT (1 MES / 30 DÍAS + EXTENSIONES)</t>
   </si>
@@ -978,19 +978,37 @@
     <t>v1.9.0</t>
   </si>
   <si>
-    <t>src/components/CertificateVerifierModal.jsx, SenceCalculatorModal.jsx, lms/views/CourseClassroomView.jsx</t>
-  </si>
-  <si>
-    <t>Nuevas Features / LMS &amp; B2B</t>
-  </si>
-  <si>
-    <t>Implementación del Verificador Público de Certificados OS-10 con QR, Simulador de Franquicia SENCE 100% y Cotizador Formal PDF para empresas, y Aula Virtual interactiva con reproductor de clases, temarios y simulador de examen teórico OS-10.</t>
-  </si>
-  <si>
-    <t>Aumentar la conversión comercial B2B, dar validación legal inmediata a egresados y enriquecer la experiencia educativa del estudiante en el campus virtual.</t>
-  </si>
-  <si>
-    <t>Plataforma líder en el norte de Chile con verificación en tiempo real, autoservicio corporativo y aula virtual interactiva.</t>
+    <t>src/lms/views/CourseClassroomView.jsx, lms/LMSLayout.jsx</t>
+  </si>
+  <si>
+    <t>Aula Virtual &amp; LMS</t>
+  </si>
+  <si>
+    <t>Implementación del Aula Virtual interactiva con reproductor de clases, temarios modulares y simulador de examen teórico OS-10.</t>
+  </si>
+  <si>
+    <t>Enriquecer la experiencia de estudio interactivo para el alumno.</t>
+  </si>
+  <si>
+    <t>Mayor retención y preparación efectiva para el examen OS-10.</t>
+  </si>
+  <si>
+    <t>v1.9.1</t>
+  </si>
+  <si>
+    <t>src/components/SenceTramosSection.jsx, lms/views/CertificateApprovalView.jsx, PersonalAreaView.jsx</t>
+  </si>
+  <si>
+    <t>Workflow &amp; Certificación</t>
+  </si>
+  <si>
+    <t>Integración en portada de Tramos de Franquicia SENCE (100%, 50%, 15% y Pago Directo por UTM). Creación del panel de Visto Bueno Administrativo para emisión de diplomas oficiales y entrega de copia digital al estudiante sin notas confidenciales.</t>
+  </si>
+  <si>
+    <t>Ajustar la visibilidad de beneficios SENCE en portada y asegurar el control administrativo de diplomas con estricta confidencialidad de notas.</t>
+  </si>
+  <si>
+    <t>Flujo administrativo formal, confidencialidad resguardada y visualización clara de tramos tributarios en la web.</t>
   </si>
   <si>
     <t>v2.0.0 (Futuro)</t>
@@ -5350,7 +5368,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -5666,7 +5684,7 @@
         <v>319</v>
       </c>
       <c r="B14" s="71" t="s">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C14" s="70" t="s">
         <v>320</v>
@@ -5683,8 +5701,34 @@
       <c r="G14" s="70" t="s">
         <v>324</v>
       </c>
-      <c r="H14" s="78" t="s">
+      <c r="H14" s="72" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="77" t="s">
         <v>325</v>
+      </c>
+      <c r="B15" s="74" t="s">
+        <v>241</v>
+      </c>
+      <c r="C15" s="73" t="s">
+        <v>326</v>
+      </c>
+      <c r="D15" s="74" t="s">
+        <v>327</v>
+      </c>
+      <c r="E15" s="73" t="s">
+        <v>328</v>
+      </c>
+      <c r="F15" s="73" t="s">
+        <v>329</v>
+      </c>
+      <c r="G15" s="73" t="s">
+        <v>330</v>
+      </c>
+      <c r="H15" s="78" t="s">
+        <v>331</v>
       </c>
     </row>
   </sheetData>
@@ -5711,7 +5755,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="67" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="B1" s="67"/>
       <c r="C1" s="67"/>
@@ -5721,104 +5765,104 @@
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="79" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="B3" s="79" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="C3" s="79" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="D3" s="79" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="E3" s="79" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="80" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="B4" s="81" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="C4" s="70" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D4" s="70" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="E4" s="70" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="82" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="B5" s="83" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="C5" s="73" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="D5" s="73" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="E5" s="73" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="80" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="B6" s="81" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="C6" s="70" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="D6" s="70" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="82" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="B7" s="83" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="C7" s="73" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="D7" s="73" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="E7" s="73" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="80" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="B8" s="81" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="C8" s="70" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="D8" s="70" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="E8" s="70" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: incorporar despacho automatico de diploma por correo al dar visto bueno con marcadores CORREO REMITENTE y CORREO DE RECEPCION
</commit_message>
<xml_diff>
--- a/Carta_Gantt_PrevySeg_2026.xlsx
+++ b/Carta_Gantt_PrevySeg_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="369">
   <si>
     <t>PREVYSEG 2026 — CRONOGRAMA MAESTRO Y CARTA GANTT (1 MES / 30 DÍAS + EXTENSIONES)</t>
   </si>
@@ -1009,6 +1009,24 @@
   </si>
   <si>
     <t>Flujo administrativo formal, confidencialidad resguardada y visualización clara de tramos tributarios en la web.</t>
+  </si>
+  <si>
+    <t>v1.9.2</t>
+  </si>
+  <si>
+    <t>src/lms/views/CertificateApprovalView.jsx</t>
+  </si>
+  <si>
+    <t>Notificación &amp; Email Dispatch</t>
+  </si>
+  <si>
+    <t>Integración del despacho automático de correo electrónico al otorgar el visto bueno administrativo del diploma con estructura ///CORREO REMITENTE/// y ///CORREO DE RECEPCION/// para enlace automático a base de datos.</t>
+  </si>
+  <si>
+    <t>Asegurar que el estudiante reciba de inmediato su copia oficial digital en su casilla de correo personal.</t>
+  </si>
+  <si>
+    <t>Entrega omnicanal de certificados (plataforma + email) y trazabilidad completa para la administración.</t>
   </si>
   <si>
     <t>v2.0.0 (Futuro)</t>
@@ -5368,7 +5386,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -5710,7 +5728,7 @@
         <v>325</v>
       </c>
       <c r="B15" s="74" t="s">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C15" s="73" t="s">
         <v>326</v>
@@ -5727,8 +5745,34 @@
       <c r="G15" s="73" t="s">
         <v>330</v>
       </c>
-      <c r="H15" s="78" t="s">
+      <c r="H15" s="72" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="76" t="s">
         <v>331</v>
+      </c>
+      <c r="B16" s="71" t="s">
+        <v>241</v>
+      </c>
+      <c r="C16" s="70" t="s">
+        <v>332</v>
+      </c>
+      <c r="D16" s="71" t="s">
+        <v>333</v>
+      </c>
+      <c r="E16" s="70" t="s">
+        <v>334</v>
+      </c>
+      <c r="F16" s="70" t="s">
+        <v>335</v>
+      </c>
+      <c r="G16" s="70" t="s">
+        <v>336</v>
+      </c>
+      <c r="H16" s="78" t="s">
+        <v>337</v>
       </c>
     </row>
   </sheetData>
@@ -5755,7 +5799,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="67" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="B1" s="67"/>
       <c r="C1" s="67"/>
@@ -5765,104 +5809,104 @@
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="79" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="B3" s="79" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="C3" s="79" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="D3" s="79" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="E3" s="79" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="80" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="B4" s="81" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="C4" s="70" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D4" s="70" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E4" s="70" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="82" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="B5" s="83" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="C5" s="73" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="D5" s="73" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="E5" s="73" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="80" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="B6" s="81" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="C6" s="70" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="D6" s="70" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="82" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="B7" s="83" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="C7" s="73" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="D7" s="73" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="E7" s="73" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="80" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="B8" s="81" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="C8" s="70" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="D8" s="70" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="E8" s="70" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: generar documento Word ERS con todos los requerimientos funcionales y no funcionales de PrevySeg con portada institucional
</commit_message>
<xml_diff>
--- a/Carta_Gantt_PrevySeg_2026.xlsx
+++ b/Carta_Gantt_PrevySeg_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="375">
   <si>
     <t>PREVYSEG 2026 — CRONOGRAMA MAESTRO Y CARTA GANTT (1 MES / 30 DÍAS + EXTENSIONES)</t>
   </si>
@@ -1027,6 +1027,24 @@
   </si>
   <si>
     <t>Entrega omnicanal de certificados (plataforma + email) y trazabilidad completa para la administración.</t>
+  </si>
+  <si>
+    <t>v1.9.3</t>
+  </si>
+  <si>
+    <t>Requerimientos_Funcionales_y_No_Funcionales_PrevySeg.docx</t>
+  </si>
+  <si>
+    <t>Documentación &amp; Ingeniería de Software</t>
+  </si>
+  <si>
+    <t>Generación del Documento Formal de Especificación de Requerimientos de Software (ERS / SRS) en formato Word (.docx) con portada institucional PrevySeg, matriz de 17 Requerimientos Funcionales (RF) y 12 Requerimientos No Funcionales (RNF) alineados a SENCE, OS-10 y NCh 2728.</t>
+  </si>
+  <si>
+    <t>Formalizar los requerimientos técnicos y funcionales de la plataforma para auditoría, desarrollo y certificación.</t>
+  </si>
+  <si>
+    <t>Documentación de ingeniería de software formal y completa para el cliente y dirección académica.</t>
   </si>
   <si>
     <t>v2.0.0 (Futuro)</t>
@@ -5386,7 +5404,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -5754,7 +5772,7 @@
         <v>331</v>
       </c>
       <c r="B16" s="71" t="s">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C16" s="70" t="s">
         <v>332</v>
@@ -5771,8 +5789,34 @@
       <c r="G16" s="70" t="s">
         <v>336</v>
       </c>
-      <c r="H16" s="78" t="s">
+      <c r="H16" s="72" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="77" t="s">
         <v>337</v>
+      </c>
+      <c r="B17" s="74" t="s">
+        <v>241</v>
+      </c>
+      <c r="C17" s="73" t="s">
+        <v>338</v>
+      </c>
+      <c r="D17" s="74" t="s">
+        <v>339</v>
+      </c>
+      <c r="E17" s="73" t="s">
+        <v>340</v>
+      </c>
+      <c r="F17" s="73" t="s">
+        <v>341</v>
+      </c>
+      <c r="G17" s="73" t="s">
+        <v>342</v>
+      </c>
+      <c r="H17" s="78" t="s">
+        <v>343</v>
       </c>
     </row>
   </sheetData>
@@ -5799,7 +5843,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="67" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="B1" s="67"/>
       <c r="C1" s="67"/>
@@ -5809,104 +5853,104 @@
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="79" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="B3" s="79" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="C3" s="79" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="D3" s="79" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="E3" s="79" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="80" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="B4" s="81" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="C4" s="70" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="D4" s="70" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="E4" s="70" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="82" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="B5" s="83" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="C5" s="73" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="D5" s="73" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="E5" s="73" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="80" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="B6" s="81" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="C6" s="70" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="D6" s="70" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="82" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="B7" s="83" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="C7" s="73" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="D7" s="73" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="E7" s="73" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="80" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="B8" s="81" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="C8" s="70" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="D8" s="70" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="E8" s="70" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: depurar catalogo a los 6 cursos activos autorizados y sincronizar en toda la plataforma
</commit_message>
<xml_diff>
--- a/Carta_Gantt_PrevySeg_2026.xlsx
+++ b/Carta_Gantt_PrevySeg_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="381">
   <si>
     <t>PREVYSEG 2026 — CRONOGRAMA MAESTRO Y CARTA GANTT (1 MES / 30 DÍAS + EXTENSIONES)</t>
   </si>
@@ -1045,6 +1045,24 @@
   </si>
   <si>
     <t>Documentación de ingeniería de software formal y completa para el cliente y dirección académica.</t>
+  </si>
+  <si>
+    <t>v1.9.4</t>
+  </si>
+  <si>
+    <t>src/components/Services.jsx, Modals.jsx, lms/views/ExtraCoursesView.jsx</t>
+  </si>
+  <si>
+    <t>Catálogo &amp; Oferta Académica</t>
+  </si>
+  <si>
+    <t>Depuración y actualización de la oferta académica a los 6 cursos activos autorizados (Resolución de Conflictos, Operador CCTV, Guardia de Seguridad, Supervisor ONLINE, Capacitación ITIC y Asistencia Curso), eliminando programas descartados.</t>
+  </si>
+  <si>
+    <t>Mantener la plataforma alineada exclusivamente con los programas vigentes y activos de PrevySeg.</t>
+  </si>
+  <si>
+    <t>Catálogo 100% conciso, filtros optimizados y consistencia en buscador y modals.</t>
   </si>
   <si>
     <t>v2.0.0 (Futuro)</t>
@@ -5404,7 +5422,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -5798,7 +5816,7 @@
         <v>337</v>
       </c>
       <c r="B17" s="74" t="s">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C17" s="73" t="s">
         <v>338</v>
@@ -5815,8 +5833,34 @@
       <c r="G17" s="73" t="s">
         <v>342</v>
       </c>
-      <c r="H17" s="78" t="s">
+      <c r="H17" s="72" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="76" t="s">
         <v>343</v>
+      </c>
+      <c r="B18" s="71" t="s">
+        <v>241</v>
+      </c>
+      <c r="C18" s="70" t="s">
+        <v>344</v>
+      </c>
+      <c r="D18" s="71" t="s">
+        <v>345</v>
+      </c>
+      <c r="E18" s="70" t="s">
+        <v>346</v>
+      </c>
+      <c r="F18" s="70" t="s">
+        <v>347</v>
+      </c>
+      <c r="G18" s="70" t="s">
+        <v>348</v>
+      </c>
+      <c r="H18" s="78" t="s">
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -5843,7 +5887,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="67" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="B1" s="67"/>
       <c r="C1" s="67"/>
@@ -5853,104 +5897,104 @@
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="79" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="B3" s="79" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="C3" s="79" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="D3" s="79" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="E3" s="79" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="80" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B4" s="81" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="C4" s="70" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="D4" s="70" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="E4" s="70" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="82" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="B5" s="83" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="C5" s="73" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="D5" s="73" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="E5" s="73" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="80" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="B6" s="81" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="C6" s="70" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="D6" s="70" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="82" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="B7" s="83" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="C7" s="73" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="D7" s="73" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="E7" s="73" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="80" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="B8" s="81" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="C8" s="70" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="D8" s="70" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="E8" s="70" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ui): refinar diseno visual con Framer Motion, glassmorphism, microinteracciones y skeleton loaders en sitio publico y LMS
</commit_message>
<xml_diff>
--- a/Carta_Gantt_PrevySeg_2026.xlsx
+++ b/Carta_Gantt_PrevySeg_2026.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="261">
   <si>
     <t>PREVYSEG 2026 — CRONOGRAMA MAESTRO Y CARTA GANTT OFICIAL (30 DÍAS / 4 SEMANAS)</t>
   </si>
@@ -186,15 +186,15 @@
     <t>PM / Fullstack</t>
   </si>
   <si>
+    <t>Mon Sep 07 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
+  </si>
+  <si>
     <t>Completado</t>
   </si>
   <si>
     <t>⭐</t>
   </si>
   <si>
-    <t>1.1</t>
-  </si>
-  <si>
     <t>Planificación</t>
   </si>
   <si>
@@ -204,7 +204,10 @@
     <t>Analista / PM</t>
   </si>
   <si>
-    <t>1.2</t>
+    <t>Tue Sep 01 2026 00:00:00 GMT-0400 (Chile Standard Time)</t>
+  </si>
+  <si>
+    <t>Wed Sep 02 2026 00:00:00 GMT-0400 (Chile Standard Time)</t>
   </si>
   <si>
     <t>Setup Inicial</t>
@@ -216,7 +219,7 @@
     <t>Dev Frontend</t>
   </si>
   <si>
-    <t>1.3</t>
+    <t>Thu Sep 03 2026 00:00:00 GMT-0400 (Chile Standard Time)</t>
   </si>
   <si>
     <t>Landing Page</t>
@@ -225,7 +228,7 @@
     <t>Hero Section con propuesta de valor, badges y llamados a la acción</t>
   </si>
   <si>
-    <t>1.4</t>
+    <t>Fri Sep 04 2026 00:00:00 GMT-0400 (Chile Standard Time)</t>
   </si>
   <si>
     <t>Catálogo Cursos</t>
@@ -234,7 +237,7 @@
     <t>Catálogo de 6 Cursos Activos con portadas Moodle y aranceles al pie</t>
   </si>
   <si>
-    <t>1.5</t>
+    <t>Sat Sep 05 2026 00:00:00 GMT-0400 (Chile Standard Time)</t>
   </si>
   <si>
     <t>Contacto Móvil</t>
@@ -246,7 +249,7 @@
     <t>Fullstack Dev</t>
   </si>
   <si>
-    <t>1.6</t>
+    <t>Sun Sep 06 2026 01:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Búsqueda &amp; UI</t>
@@ -270,7 +273,7 @@
     <t>⭐ HITO 2: Campus Virtual LMS y Espacio del Estudiante Operativo</t>
   </si>
   <si>
-    <t>2.1</t>
+    <t>Mon Sep 14 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Seguridad / Auth</t>
@@ -279,7 +282,10 @@
     <t>Sistema de Autenticación con RUT y Password (RBAC Student / Admin)</t>
   </si>
   <si>
-    <t>2.2</t>
+    <t>Tue Sep 08 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
+  </si>
+  <si>
+    <t>Thu Sep 10 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>LMS Layout</t>
@@ -288,7 +294,10 @@
     <t>Estructura LMSLayout con Topbar, navegación lateral y badges SENCE</t>
   </si>
   <si>
-    <t>2.3</t>
+    <t>Wed Sep 09 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
+  </si>
+  <si>
+    <t>Fri Sep 11 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Área Personal</t>
@@ -297,7 +306,7 @@
     <t>Área Personal del Estudiante con Línea de Tiempo y seguimiento de avance</t>
   </si>
   <si>
-    <t>2.4</t>
+    <t>Sat Sep 12 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Mis Cursos</t>
@@ -306,7 +315,7 @@
     <t>Vista Mis Cursos con tarjetas de progreso curricular e inicio de clases</t>
   </si>
   <si>
-    <t>2.5</t>
+    <t>Sun Sep 13 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Gestión Inicial</t>
@@ -327,7 +336,7 @@
     <t>⭐ HITO 3: Aula Virtual Interactiva y Servicios Académicos Completos</t>
   </si>
   <si>
-    <t>3.1</t>
+    <t>Mon Sep 21 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Aula Virtual</t>
@@ -336,7 +345,10 @@
     <t>Reproductor de Video de Clases HD con avance porcentual por lección</t>
   </si>
   <si>
-    <t>3.2</t>
+    <t>Tue Sep 15 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
+  </si>
+  <si>
+    <t>Thu Sep 17 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Temario Acordeón</t>
@@ -345,7 +357,10 @@
     <t>Estructura modular de 4 módulos con contenidos teóricos y prácticos</t>
   </si>
   <si>
-    <t>3.3</t>
+    <t>Wed Sep 16 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Evaluación OS-10</t>
@@ -354,7 +369,7 @@
     <t>Simulador de Examen Teórico OS-10 con temporizador y retroalimentación</t>
   </si>
   <si>
-    <t>3.4</t>
+    <t>Sat Sep 19 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Fidelización</t>
@@ -363,7 +378,7 @@
     <t>Catálogo de Capacitaciones Extras con 15% de descuento exclusivo alumno</t>
   </si>
   <si>
-    <t>3.5</t>
+    <t>Sun Sep 20 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Intermediación</t>
@@ -387,7 +402,7 @@
     <t>PM / Arquitecto</t>
   </si>
   <si>
-    <t>4.1</t>
+    <t>Wed Sep 30 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Visto Bueno Admin</t>
@@ -396,7 +411,10 @@
     <t>Panel de Verificación y Visto Bueno Administrativo para Emisión de Diplomas</t>
   </si>
   <si>
-    <t>4.2</t>
+    <t>Tue Sep 22 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
+  </si>
+  <si>
+    <t>Thu Sep 24 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Despacho Correo</t>
@@ -405,7 +423,7 @@
     <t>Despacho Automático de Diploma PDF (///CORREO REMITENTE/// -&gt; ///CORREO DE RECEPCION///)</t>
   </si>
   <si>
-    <t>4.3</t>
+    <t>Sat Sep 26 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Confidencialidad</t>
@@ -414,7 +432,10 @@
     <t>Copia Oficial para el Alumno en PDF acreditando idoneidad (Sin notas numéricas)</t>
   </si>
   <si>
-    <t>4.4</t>
+    <t>Fri Sep 25 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
+  </si>
+  <si>
+    <t>Sun Sep 27 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Franquicia SENCE</t>
@@ -423,7 +444,7 @@
     <t>Sección de Tramos de Franquicia SENCE (100%, 50%, 15% y Pago Directo por UTM)</t>
   </si>
   <si>
-    <t>4.5</t>
+    <t>Mon Sep 28 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Documentación ERS</t>
@@ -435,7 +456,7 @@
     <t>PM / QA</t>
   </si>
   <si>
-    <t>4.6</t>
+    <t>Tue Sep 29 2026 00:00:00 GMT-0300 (Chile Summer Time)</t>
   </si>
   <si>
     <t>Despliegue GitHub</t>
@@ -782,9 +803,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="164" formatCode="yyyy/m/d"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -794,68 +815,72 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="15"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <i/>
-      <color rgb="E2E8F0"/>
-      <sz val="10.5"/>
+      <color rgb="FFE2E8F0"/>
+      <sz val="10"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="0F172A"/>
+      <color rgb="FF0F172A"/>
       <sz val="10"/>
       <name val="Segoe UI"/>
     </font>
     <font>
-      <color rgb="475569"/>
-      <sz val="8.5"/>
+      <color rgb="FF475569"/>
+      <sz val="8"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="2563EB"/>
+      <color rgb="FF2563EB"/>
       <sz val="13"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="16A34A"/>
+      <color rgb="FF16A34A"/>
       <sz val="13"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="0284C7"/>
+      <color rgb="FF0284C7"/>
       <sz val="12"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFF"/>
-      <sz val="9.5"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="334155"/>
+      <color rgb="FF334155"/>
       <sz val="8"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="78350F"/>
-      <sz val="8.5"/>
+      <color rgb="FF78350F"/>
+      <sz val="8"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="166534"/>
-      <sz val="8.5"/>
+      <color rgb="FF166534"/>
+      <sz val="8"/>
       <name val="Segoe UI"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
@@ -863,37 +888,37 @@
       <name val="Segoe UI"/>
     </font>
     <font>
-      <color rgb="1E293B"/>
-      <sz val="8.5"/>
+      <color rgb="FF1E293B"/>
+      <sz val="8"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="D97706"/>
-      <sz val="9.5"/>
+      <color rgb="FFD97706"/>
+      <sz val="9"/>
       <name val="Segoe UI"/>
     </font>
     <font>
-      <color rgb="1E293B"/>
+      <color rgb="FF1E293B"/>
       <sz val="9"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="166534"/>
+      <color rgb="FF166534"/>
       <sz val="9"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
-      <color rgb="2563EB"/>
-      <sz val="9.5"/>
+      <color rgb="FF2563EB"/>
+      <sz val="9"/>
       <name val="Segoe UI"/>
     </font>
   </fonts>
@@ -906,87 +931,87 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0F172A"/>
+        <fgColor rgb="FF0F172A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="1E293B"/>
+        <fgColor rgb="FF1E293B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="F8FAFC"/>
+        <fgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="1E3A8A"/>
+        <fgColor rgb="FF1E3A8A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="1D4ED8"/>
+        <fgColor rgb="FF1D4ED8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="2563EB"/>
+        <fgColor rgb="FF2563EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="3B82F6"/>
+        <fgColor rgb="FF3B82F6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="E2E8F0"/>
+        <fgColor rgb="FFE2E8F0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="F1F5F9"/>
+        <fgColor rgb="FFF1F5F9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FEF3C7"/>
+        <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="DCFCE7"/>
+        <fgColor rgb="FFDCFCE7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="F59E0B"/>
+        <fgColor rgb="FFF59E0B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="86EFAC"/>
+        <fgColor rgb="FF86EFAC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="7DD3FC"/>
+        <fgColor rgb="FF7DD3FC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="93C5FD"/>
+        <fgColor rgb="FF93C5FD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="6EE7B7"/>
+        <fgColor rgb="FF6EE7B7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="EFF6FF"/>
+        <fgColor rgb="FFEFF6FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -1000,31 +1025,31 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </left>
       <right style="thin">
-        <color rgb="CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </right>
       <top style="thin">
-        <color rgb="CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </top>
       <bottom style="thin">
-        <color rgb="CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="334155"/>
+        <color rgb="FF334155"/>
       </left>
       <right style="thin">
-        <color rgb="334155"/>
+        <color rgb="FF334155"/>
       </right>
       <top style="medium">
-        <color rgb="0F172A"/>
+        <color rgb="FF0F172A"/>
       </top>
       <bottom style="medium">
-        <color rgb="0F172A"/>
+        <color rgb="FF0F172A"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1077,7 +1102,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" indent="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1088,82 +1113,82 @@
     <xf numFmtId="164" fontId="10" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="10" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="10" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1508,18 +1533,19 @@
   <dimension ref="A1:AN38"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="7" customWidth="1"/>
+    <col min="1" max="1" width="9.285714285714286" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="3" max="3" width="42.142857142857146" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="6" customWidth="1"/>
+    <col min="7" max="7" width="9.285714285714286" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="39" width="4" customWidth="1"/>
+    <col min="10" max="39" width="9.285714285714286" customWidth="1"/>
+    <col min="40" max="40" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="1" ht="32.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1563,7 +1589,7 @@
       <c r="AM1" s="1"/>
       <c r="AN1" s="1"/>
     </row>
-    <row r="2" ht="20" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="2" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1647,7 +1673,7 @@
       </c>
       <c r="J5" s="6"/>
     </row>
-    <row r="7" ht="22" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="7" ht="21.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1815,7 +1841,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="9" ht="21.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
         <v>52</v>
       </c>
@@ -1859,7 +1885,7 @@
       <c r="AM9" s="15"/>
       <c r="AN9" s="15"/>
     </row>
-    <row r="10" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="10" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
         <v>53</v>
       </c>
@@ -1872,11 +1898,11 @@
       <c r="D10" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="E10" s="18">
-        <v>46272.125</v>
-      </c>
-      <c r="F10" s="18">
-        <v>46272.125</v>
+      <c r="E10" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" s="18" t="s">
+        <v>57</v>
       </c>
       <c r="G10" s="16">
         <v>1</v>
@@ -1885,7 +1911,7 @@
         <v>1</v>
       </c>
       <c r="I10" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J10" s="21"/>
       <c r="K10" s="21"/>
@@ -1894,7 +1920,7 @@
       <c r="N10" s="21"/>
       <c r="O10" s="22"/>
       <c r="P10" s="23" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q10" s="21"/>
       <c r="R10" s="21"/>
@@ -1920,9 +1946,9 @@
       <c r="AL10" s="21"/>
       <c r="AM10" s="21"/>
     </row>
-    <row r="11" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A11" s="24" t="s">
-        <v>59</v>
+    <row r="11" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A11" s="24">
+        <v>1.1</v>
       </c>
       <c r="B11" s="25" t="s">
         <v>60</v>
@@ -1933,11 +1959,11 @@
       <c r="D11" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="E11" s="26">
-        <v>46266.16666666667</v>
-      </c>
-      <c r="F11" s="26">
-        <v>46267.16666666667</v>
+      <c r="E11" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="F11" s="26" t="s">
+        <v>64</v>
       </c>
       <c r="G11" s="24">
         <v>2</v>
@@ -1946,7 +1972,7 @@
         <v>1</v>
       </c>
       <c r="I11" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J11" s="28"/>
       <c r="K11" s="28"/>
@@ -1979,24 +2005,24 @@
       <c r="AL11" s="21"/>
       <c r="AM11" s="21"/>
     </row>
-    <row r="12" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A12" s="29" t="s">
+    <row r="12" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A12" s="29">
+        <v>1.2</v>
+      </c>
+      <c r="B12" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="B12" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="E12" s="31">
-        <v>46266.16666666667</v>
-      </c>
-      <c r="F12" s="31">
-        <v>46268.16666666667</v>
+      <c r="F12" s="31" t="s">
+        <v>68</v>
       </c>
       <c r="G12" s="29">
         <v>3</v>
@@ -2005,7 +2031,7 @@
         <v>1</v>
       </c>
       <c r="I12" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J12" s="28"/>
       <c r="K12" s="28"/>
@@ -2038,24 +2064,24 @@
       <c r="AL12" s="21"/>
       <c r="AM12" s="21"/>
     </row>
-    <row r="13" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A13" s="24" t="s">
+    <row r="13" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A13" s="24">
+        <v>1.3</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="D13" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="B13" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="C13" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="D13" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="E13" s="26">
-        <v>46267.16666666667</v>
-      </c>
-      <c r="F13" s="26">
-        <v>46269.16666666667</v>
+      <c r="E13" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="F13" s="26" t="s">
+        <v>71</v>
       </c>
       <c r="G13" s="24">
         <v>3</v>
@@ -2064,7 +2090,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J13" s="21"/>
       <c r="K13" s="28"/>
@@ -2097,24 +2123,24 @@
       <c r="AL13" s="21"/>
       <c r="AM13" s="21"/>
     </row>
-    <row r="14" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A14" s="29" t="s">
-        <v>70</v>
+    <row r="14" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A14" s="29">
+        <v>1.4</v>
       </c>
       <c r="B14" s="30" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C14" s="30" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="E14" s="31">
-        <v>46268.16666666667</v>
-      </c>
-      <c r="F14" s="31">
-        <v>46270.16666666667</v>
+        <v>67</v>
+      </c>
+      <c r="E14" s="31" t="s">
+        <v>68</v>
+      </c>
+      <c r="F14" s="31" t="s">
+        <v>74</v>
       </c>
       <c r="G14" s="29">
         <v>3</v>
@@ -2123,7 +2149,7 @@
         <v>1</v>
       </c>
       <c r="I14" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J14" s="21"/>
       <c r="K14" s="21"/>
@@ -2156,24 +2182,24 @@
       <c r="AL14" s="21"/>
       <c r="AM14" s="21"/>
     </row>
-    <row r="15" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A15" s="24" t="s">
-        <v>73</v>
+    <row r="15" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A15" s="24">
+        <v>1.5</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D15" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="E15" s="26">
-        <v>46269.16666666667</v>
-      </c>
-      <c r="F15" s="26">
-        <v>46271.16666666667</v>
+        <v>77</v>
+      </c>
+      <c r="E15" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="F15" s="26" t="s">
+        <v>78</v>
       </c>
       <c r="G15" s="24">
         <v>3</v>
@@ -2182,7 +2208,7 @@
         <v>1</v>
       </c>
       <c r="I15" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J15" s="21"/>
       <c r="K15" s="21"/>
@@ -2215,24 +2241,24 @@
       <c r="AL15" s="21"/>
       <c r="AM15" s="21"/>
     </row>
-    <row r="16" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A16" s="29" t="s">
-        <v>77</v>
+    <row r="16" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A16" s="29">
+        <v>1.6</v>
       </c>
       <c r="B16" s="30" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D16" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="E16" s="31">
-        <v>46270.16666666667</v>
-      </c>
-      <c r="F16" s="31">
-        <v>46272.125</v>
+        <v>81</v>
+      </c>
+      <c r="E16" s="31" t="s">
+        <v>74</v>
+      </c>
+      <c r="F16" s="31" t="s">
+        <v>57</v>
       </c>
       <c r="G16" s="29">
         <v>3</v>
@@ -2241,7 +2267,7 @@
         <v>1</v>
       </c>
       <c r="I16" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J16" s="21"/>
       <c r="K16" s="21"/>
@@ -2274,9 +2300,9 @@
       <c r="AL16" s="21"/>
       <c r="AM16" s="21"/>
     </row>
-    <row r="17" ht="22" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="17" ht="21.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A17" s="33" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B17" s="33"/>
       <c r="C17" s="33"/>
@@ -2318,24 +2344,24 @@
       <c r="AM17" s="33"/>
       <c r="AN17" s="33"/>
     </row>
-    <row r="18" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="18" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D18" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="E18" s="18">
-        <v>46279.125</v>
-      </c>
-      <c r="F18" s="18">
-        <v>46279.125</v>
+      <c r="E18" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>86</v>
       </c>
       <c r="G18" s="16">
         <v>1</v>
@@ -2344,7 +2370,7 @@
         <v>1</v>
       </c>
       <c r="I18" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J18" s="21"/>
       <c r="K18" s="21"/>
@@ -2360,7 +2386,7 @@
       <c r="U18" s="21"/>
       <c r="V18" s="22"/>
       <c r="W18" s="23" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="X18" s="21"/>
       <c r="Y18" s="21"/>
@@ -2379,24 +2405,24 @@
       <c r="AL18" s="21"/>
       <c r="AM18" s="21"/>
     </row>
-    <row r="19" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A19" s="24" t="s">
-        <v>85</v>
+    <row r="19" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A19" s="24">
+        <v>2.1</v>
       </c>
       <c r="B19" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D19" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="E19" s="26">
-        <v>46273.125</v>
-      </c>
-      <c r="F19" s="26">
-        <v>46275.125</v>
+        <v>77</v>
+      </c>
+      <c r="E19" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="F19" s="26" t="s">
+        <v>90</v>
       </c>
       <c r="G19" s="24">
         <v>3</v>
@@ -2405,7 +2431,7 @@
         <v>1</v>
       </c>
       <c r="I19" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J19" s="21"/>
       <c r="K19" s="21"/>
@@ -2438,24 +2464,24 @@
       <c r="AL19" s="21"/>
       <c r="AM19" s="21"/>
     </row>
-    <row r="20" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A20" s="29" t="s">
-        <v>88</v>
+    <row r="20" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A20" s="29">
+        <v>2.2</v>
       </c>
       <c r="B20" s="30" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C20" s="30" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D20" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="E20" s="31">
-        <v>46274.125</v>
-      </c>
-      <c r="F20" s="31">
-        <v>46276.125</v>
+        <v>67</v>
+      </c>
+      <c r="E20" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="F20" s="31" t="s">
+        <v>94</v>
       </c>
       <c r="G20" s="29">
         <v>3</v>
@@ -2464,7 +2490,7 @@
         <v>1</v>
       </c>
       <c r="I20" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J20" s="21"/>
       <c r="K20" s="21"/>
@@ -2497,24 +2523,24 @@
       <c r="AL20" s="21"/>
       <c r="AM20" s="21"/>
     </row>
-    <row r="21" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A21" s="24" t="s">
-        <v>91</v>
+    <row r="21" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A21" s="24">
+        <v>2.3</v>
       </c>
       <c r="B21" s="25" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D21" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="E21" s="26">
-        <v>46275.125</v>
-      </c>
-      <c r="F21" s="26">
-        <v>46277.125</v>
+        <v>67</v>
+      </c>
+      <c r="E21" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="26" t="s">
+        <v>97</v>
       </c>
       <c r="G21" s="24">
         <v>3</v>
@@ -2523,7 +2549,7 @@
         <v>1</v>
       </c>
       <c r="I21" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J21" s="21"/>
       <c r="K21" s="21"/>
@@ -2556,24 +2582,24 @@
       <c r="AL21" s="21"/>
       <c r="AM21" s="21"/>
     </row>
-    <row r="22" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A22" s="29" t="s">
+    <row r="22" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A22" s="29">
+        <v>2.4</v>
+      </c>
+      <c r="B22" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="D22" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="E22" s="31" t="s">
         <v>94</v>
       </c>
-      <c r="B22" s="30" t="s">
-        <v>95</v>
-      </c>
-      <c r="C22" s="30" t="s">
-        <v>96</v>
-      </c>
-      <c r="D22" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="E22" s="31">
-        <v>46276.125</v>
-      </c>
-      <c r="F22" s="31">
-        <v>46278.125</v>
+      <c r="F22" s="31" t="s">
+        <v>100</v>
       </c>
       <c r="G22" s="29">
         <v>3</v>
@@ -2582,7 +2608,7 @@
         <v>1</v>
       </c>
       <c r="I22" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J22" s="21"/>
       <c r="K22" s="21"/>
@@ -2615,24 +2641,24 @@
       <c r="AL22" s="21"/>
       <c r="AM22" s="21"/>
     </row>
-    <row r="23" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A23" s="24" t="s">
+    <row r="23" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A23" s="24">
+        <v>2.5</v>
+      </c>
+      <c r="B23" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="C23" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="D23" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="E23" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="B23" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="C23" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="D23" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="E23" s="26">
-        <v>46277.125</v>
-      </c>
-      <c r="F23" s="26">
-        <v>46279.125</v>
+      <c r="F23" s="26" t="s">
+        <v>86</v>
       </c>
       <c r="G23" s="24">
         <v>3</v>
@@ -2641,7 +2667,7 @@
         <v>1</v>
       </c>
       <c r="I23" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J23" s="21"/>
       <c r="K23" s="21"/>
@@ -2674,9 +2700,9 @@
       <c r="AL23" s="21"/>
       <c r="AM23" s="21"/>
     </row>
-    <row r="24" ht="22" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="24" ht="21.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A24" s="35" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B24" s="35"/>
       <c r="C24" s="35"/>
@@ -2718,24 +2744,24 @@
       <c r="AM24" s="35"/>
       <c r="AN24" s="35"/>
     </row>
-    <row r="25" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="25" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D25" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="E25" s="18">
-        <v>46286.125</v>
-      </c>
-      <c r="F25" s="18">
-        <v>46286.125</v>
+      <c r="E25" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="F25" s="18" t="s">
+        <v>107</v>
       </c>
       <c r="G25" s="16">
         <v>1</v>
@@ -2744,7 +2770,7 @@
         <v>1</v>
       </c>
       <c r="I25" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J25" s="21"/>
       <c r="K25" s="21"/>
@@ -2767,7 +2793,7 @@
       <c r="AB25" s="21"/>
       <c r="AC25" s="22"/>
       <c r="AD25" s="23" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="AE25" s="21"/>
       <c r="AF25" s="21"/>
@@ -2779,24 +2805,24 @@
       <c r="AL25" s="21"/>
       <c r="AM25" s="21"/>
     </row>
-    <row r="26" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A26" s="29" t="s">
-        <v>104</v>
+    <row r="26" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A26" s="29">
+        <v>3.1</v>
       </c>
       <c r="B26" s="30" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C26" s="30" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D26" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="E26" s="31">
-        <v>46280.125</v>
-      </c>
-      <c r="F26" s="31">
-        <v>46282.125</v>
+        <v>67</v>
+      </c>
+      <c r="E26" s="31" t="s">
+        <v>110</v>
+      </c>
+      <c r="F26" s="31" t="s">
+        <v>111</v>
       </c>
       <c r="G26" s="29">
         <v>3</v>
@@ -2805,7 +2831,7 @@
         <v>1</v>
       </c>
       <c r="I26" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J26" s="21"/>
       <c r="K26" s="21"/>
@@ -2838,24 +2864,24 @@
       <c r="AL26" s="21"/>
       <c r="AM26" s="21"/>
     </row>
-    <row r="27" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A27" s="24" t="s">
-        <v>107</v>
+    <row r="27" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A27" s="24">
+        <v>3.2</v>
       </c>
       <c r="B27" s="25" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D27" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="E27" s="26">
-        <v>46281.125</v>
-      </c>
-      <c r="F27" s="26">
-        <v>46283.125</v>
+        <v>67</v>
+      </c>
+      <c r="E27" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="F27" s="26" t="s">
+        <v>115</v>
       </c>
       <c r="G27" s="24">
         <v>3</v>
@@ -2864,7 +2890,7 @@
         <v>1</v>
       </c>
       <c r="I27" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J27" s="21"/>
       <c r="K27" s="21"/>
@@ -2897,24 +2923,24 @@
       <c r="AL27" s="21"/>
       <c r="AM27" s="21"/>
     </row>
-    <row r="28" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A28" s="29" t="s">
-        <v>110</v>
+    <row r="28" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A28" s="29">
+        <v>3.3</v>
       </c>
       <c r="B28" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="C28" s="30" t="s">
+        <v>117</v>
+      </c>
+      <c r="D28" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="E28" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="C28" s="30" t="s">
-        <v>112</v>
-      </c>
-      <c r="D28" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="E28" s="31">
-        <v>46282.125</v>
-      </c>
-      <c r="F28" s="31">
-        <v>46284.125</v>
+      <c r="F28" s="31" t="s">
+        <v>118</v>
       </c>
       <c r="G28" s="29">
         <v>3</v>
@@ -2923,7 +2949,7 @@
         <v>1</v>
       </c>
       <c r="I28" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J28" s="21"/>
       <c r="K28" s="21"/>
@@ -2956,24 +2982,24 @@
       <c r="AL28" s="21"/>
       <c r="AM28" s="21"/>
     </row>
-    <row r="29" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A29" s="24" t="s">
-        <v>113</v>
+    <row r="29" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A29" s="24">
+        <v>3.4</v>
       </c>
       <c r="B29" s="25" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C29" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="D29" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="E29" s="26" t="s">
         <v>115</v>
       </c>
-      <c r="D29" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="E29" s="26">
-        <v>46283.125</v>
-      </c>
-      <c r="F29" s="26">
-        <v>46285.125</v>
+      <c r="F29" s="26" t="s">
+        <v>121</v>
       </c>
       <c r="G29" s="24">
         <v>3</v>
@@ -2982,7 +3008,7 @@
         <v>1</v>
       </c>
       <c r="I29" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J29" s="21"/>
       <c r="K29" s="21"/>
@@ -3015,24 +3041,24 @@
       <c r="AL29" s="21"/>
       <c r="AM29" s="21"/>
     </row>
-    <row r="30" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A30" s="29" t="s">
-        <v>116</v>
+    <row r="30" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A30" s="29">
+        <v>3.5</v>
       </c>
       <c r="B30" s="30" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="C30" s="30" t="s">
+        <v>123</v>
+      </c>
+      <c r="D30" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="E30" s="31" t="s">
         <v>118</v>
       </c>
-      <c r="D30" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="E30" s="31">
-        <v>46284.125</v>
-      </c>
-      <c r="F30" s="31">
-        <v>46286.125</v>
+      <c r="F30" s="31" t="s">
+        <v>107</v>
       </c>
       <c r="G30" s="29">
         <v>3</v>
@@ -3041,7 +3067,7 @@
         <v>1</v>
       </c>
       <c r="I30" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J30" s="21"/>
       <c r="K30" s="21"/>
@@ -3074,9 +3100,9 @@
       <c r="AL30" s="21"/>
       <c r="AM30" s="21"/>
     </row>
-    <row r="31" ht="22" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="31" ht="21.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A31" s="37" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B31" s="37"/>
       <c r="C31" s="37"/>
@@ -3118,24 +3144,24 @@
       <c r="AM31" s="37"/>
       <c r="AN31" s="37"/>
     </row>
-    <row r="32" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="32" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>123</v>
-      </c>
-      <c r="E32" s="18">
-        <v>46295.125</v>
-      </c>
-      <c r="F32" s="18">
-        <v>46295.125</v>
+        <v>128</v>
+      </c>
+      <c r="E32" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="F32" s="18" t="s">
+        <v>129</v>
       </c>
       <c r="G32" s="16">
         <v>1</v>
@@ -3144,7 +3170,7 @@
         <v>1</v>
       </c>
       <c r="I32" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J32" s="21"/>
       <c r="K32" s="21"/>
@@ -3176,27 +3202,27 @@
       <c r="AK32" s="22"/>
       <c r="AL32" s="21"/>
       <c r="AM32" s="23" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="33" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A33" s="24" t="s">
-        <v>124</v>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="33" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A33" s="24">
+        <v>4.1</v>
       </c>
       <c r="B33" s="25" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C33" s="25" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D33" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="E33" s="26">
-        <v>46287.125</v>
-      </c>
-      <c r="F33" s="26">
-        <v>46289.125</v>
+        <v>77</v>
+      </c>
+      <c r="E33" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="F33" s="26" t="s">
+        <v>133</v>
       </c>
       <c r="G33" s="24">
         <v>3</v>
@@ -3205,7 +3231,7 @@
         <v>1</v>
       </c>
       <c r="I33" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J33" s="21"/>
       <c r="K33" s="21"/>
@@ -3238,24 +3264,24 @@
       <c r="AL33" s="21"/>
       <c r="AM33" s="21"/>
     </row>
-    <row r="34" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A34" s="29" t="s">
-        <v>127</v>
+    <row r="34" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A34" s="29">
+        <v>4.2</v>
       </c>
       <c r="B34" s="30" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="C34" s="30" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="D34" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="E34" s="31">
-        <v>46289.125</v>
-      </c>
-      <c r="F34" s="31">
-        <v>46291.125</v>
+        <v>77</v>
+      </c>
+      <c r="E34" s="31" t="s">
+        <v>133</v>
+      </c>
+      <c r="F34" s="31" t="s">
+        <v>136</v>
       </c>
       <c r="G34" s="29">
         <v>3</v>
@@ -3264,7 +3290,7 @@
         <v>1</v>
       </c>
       <c r="I34" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J34" s="21"/>
       <c r="K34" s="21"/>
@@ -3297,24 +3323,24 @@
       <c r="AL34" s="21"/>
       <c r="AM34" s="21"/>
     </row>
-    <row r="35" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A35" s="24" t="s">
-        <v>130</v>
+    <row r="35" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A35" s="24">
+        <v>4.3</v>
       </c>
       <c r="B35" s="25" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C35" s="25" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="D35" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="E35" s="26">
-        <v>46290.125</v>
-      </c>
-      <c r="F35" s="26">
-        <v>46292.125</v>
+        <v>67</v>
+      </c>
+      <c r="E35" s="26" t="s">
+        <v>139</v>
+      </c>
+      <c r="F35" s="26" t="s">
+        <v>140</v>
       </c>
       <c r="G35" s="24">
         <v>3</v>
@@ -3323,7 +3349,7 @@
         <v>1</v>
       </c>
       <c r="I35" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J35" s="21"/>
       <c r="K35" s="21"/>
@@ -3356,24 +3382,24 @@
       <c r="AL35" s="21"/>
       <c r="AM35" s="21"/>
     </row>
-    <row r="36" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A36" s="29" t="s">
-        <v>133</v>
+    <row r="36" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A36" s="29">
+        <v>4.4</v>
       </c>
       <c r="B36" s="30" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C36" s="30" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="D36" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="E36" s="31">
-        <v>46291.125</v>
-      </c>
-      <c r="F36" s="31">
-        <v>46293.125</v>
+        <v>67</v>
+      </c>
+      <c r="E36" s="31" t="s">
+        <v>136</v>
+      </c>
+      <c r="F36" s="31" t="s">
+        <v>143</v>
       </c>
       <c r="G36" s="29">
         <v>3</v>
@@ -3382,7 +3408,7 @@
         <v>1</v>
       </c>
       <c r="I36" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J36" s="21"/>
       <c r="K36" s="21"/>
@@ -3415,24 +3441,24 @@
       <c r="AL36" s="21"/>
       <c r="AM36" s="21"/>
     </row>
-    <row r="37" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A37" s="24" t="s">
-        <v>136</v>
+    <row r="37" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A37" s="24">
+        <v>4.5</v>
       </c>
       <c r="B37" s="25" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="D37" s="24" t="s">
-        <v>139</v>
-      </c>
-      <c r="E37" s="26">
-        <v>46293.125</v>
-      </c>
-      <c r="F37" s="26">
-        <v>46294.125</v>
+        <v>146</v>
+      </c>
+      <c r="E37" s="26" t="s">
+        <v>143</v>
+      </c>
+      <c r="F37" s="26" t="s">
+        <v>147</v>
       </c>
       <c r="G37" s="24">
         <v>2</v>
@@ -3441,7 +3467,7 @@
         <v>1</v>
       </c>
       <c r="I37" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J37" s="21"/>
       <c r="K37" s="21"/>
@@ -3474,24 +3500,24 @@
       <c r="AL37" s="38"/>
       <c r="AM37" s="21"/>
     </row>
-    <row r="38" ht="19" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A38" s="29" t="s">
-        <v>140</v>
+    <row r="38" ht="18.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A38" s="29">
+        <v>4.6</v>
       </c>
       <c r="B38" s="30" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="C38" s="30" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D38" s="29" t="s">
-        <v>143</v>
-      </c>
-      <c r="E38" s="31">
-        <v>46294.125</v>
-      </c>
-      <c r="F38" s="31">
-        <v>46295.125</v>
+        <v>150</v>
+      </c>
+      <c r="E38" s="31" t="s">
+        <v>147</v>
+      </c>
+      <c r="F38" s="31" t="s">
+        <v>129</v>
       </c>
       <c r="G38" s="29">
         <v>2</v>
@@ -3500,7 +3526,7 @@
         <v>1</v>
       </c>
       <c r="I38" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J38" s="21"/>
       <c r="K38" s="21"/>
@@ -3581,11 +3607,12 @@
     <col min="5" max="5" width="34" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
+    <col min="8" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="39" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="B1" s="39"/>
       <c r="C1" s="39"/>
@@ -3596,117 +3623,117 @@
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="F3" s="8" t="s">
         <v>17</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="40" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="B4" s="41" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="C4" s="42" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="D4" s="41" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="E4" s="41" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="F4" s="43" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G4" s="41" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="40" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C5" s="45" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D5" s="44" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="E5" s="44" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="F5" s="43" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G5" s="44" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="40" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="B6" s="41" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="C6" s="42" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="D6" s="41" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="E6" s="41" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="F6" s="43" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G6" s="41" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="40" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="B7" s="44" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C7" s="45" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="D7" s="44" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="E7" s="44" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="F7" s="43" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G7" s="44" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -3726,15 +3753,16 @@
     <col min="1" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="44" customWidth="1"/>
+    <col min="5" max="5" width="42.142857142857146" customWidth="1"/>
     <col min="6" max="6" width="32" customWidth="1"/>
     <col min="7" max="7" width="28" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="46" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -3746,25 +3774,25 @@
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="47" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="B3" s="47" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="C3" s="47" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="D3" s="47" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="E3" s="47" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="F3" s="47" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="G3" s="47" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="H3" s="47" t="s">
         <v>17</v>
@@ -3772,288 +3800,288 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="48" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="B4" s="42" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="E4" s="41" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="F4" s="41" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="G4" s="41" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="H4" s="43" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="48" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="B5" s="45" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="C5" s="44" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="D5" s="45" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="E5" s="44" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="F5" s="44" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="G5" s="44" t="s">
+        <v>203</v>
+      </c>
+      <c r="H5" s="43" t="s">
         <v>196</v>
-      </c>
-      <c r="H5" s="43" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="48" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="E6" s="41" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="F6" s="41" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="G6" s="41" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="H6" s="43" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="48" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="B7" s="45" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="C7" s="44" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="D7" s="45" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="E7" s="44" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="F7" s="44" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="G7" s="44" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="H7" s="43" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="48" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="B8" s="42" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="E8" s="41" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="F8" s="41" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="G8" s="41" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="H8" s="43" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="48" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="B9" s="45" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="C9" s="44" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="D9" s="45" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="E9" s="44" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="F9" s="44" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="G9" s="44" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="H9" s="43" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="48" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="B10" s="42" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E10" s="41" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="F10" s="41" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="G10" s="41" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="H10" s="43" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="48" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="B11" s="45" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="C11" s="44" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="D11" s="45" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="E11" s="44" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="F11" s="44" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="G11" s="44" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="H11" s="43" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="48" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="B12" s="42" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="E12" s="41" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="F12" s="41" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="G12" s="41" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="H12" s="43" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="48" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="B13" s="45" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="C13" s="44" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="D13" s="45" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="E13" s="44" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="F13" s="44" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="G13" s="44" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="H13" s="43" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="48" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="B14" s="42" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="E14" s="41" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="F14" s="41" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="G14" s="41" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="H14" s="43" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>